<commit_message>
update vtk grid helpers
</commit_message>
<xml_diff>
--- a/tests/ITER_3D_APEC_evol/input_template.xlsx
+++ b/tests/ITER_3D_APEC_evol/input_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\APEC-M\tests\ITER_2D_APEC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\APEC-M\tests\ITER_3D_APEC_evol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F11BD908-ACEB-4D4E-8982-195D3AC8E578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47328260-D5AA-4415-B92B-BFF143C48448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="element_types" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="111">
   <si>
     <t>time_step_number</t>
   </si>
@@ -359,6 +359,9 @@
   </si>
   <si>
     <t>PLANE233</t>
+  </si>
+  <si>
+    <t>SOLID97</t>
   </si>
 </sst>
 </file>
@@ -368,7 +371,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -387,6 +390,12 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -750,7 +759,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
@@ -832,7 +841,7 @@
         <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C4" s="1">
         <v>4</v>
@@ -851,14 +860,53 @@
       </c>
     </row>
     <row r="5" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
+      <c r="A5" s="1">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" s="1">
+        <v>3</v>
+      </c>
+      <c r="D5" s="1">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fixed point for refactoring
</commit_message>
<xml_diff>
--- a/tests/ITER_3D_APEC_evol/input_template.xlsx
+++ b/tests/ITER_3D_APEC_evol/input_template.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PlasmaArc\tests\ITER_3D_APEC_evol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8DD31EF-204F-4A70-9536-FA1AFC75CB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49197BFE-9D38-41E7-89B3-115792F5566E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1380" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="element_types" sheetId="1" r:id="rId1"/>
-    <sheet name="cp" sheetId="2" r:id="rId2"/>
+    <sheet name="dof_couplings" sheetId="2" r:id="rId2"/>
     <sheet name="cpcyc" sheetId="3" r:id="rId3"/>
     <sheet name="materials" sheetId="4" r:id="rId4"/>
     <sheet name="real_constants" sheetId="5" r:id="rId5"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="111">
   <si>
     <t>time_step_number</t>
   </si>
@@ -331,9 +331,6 @@
     <t>dof4</t>
   </si>
   <si>
-    <t>CP_ID</t>
-  </si>
-  <si>
     <t>ansys_etype</t>
   </si>
   <si>
@@ -359,6 +356,12 @@
   </si>
   <si>
     <t>SOLID97</t>
+  </si>
+  <si>
+    <t>cp_id</t>
+  </si>
+  <si>
+    <t>variable</t>
   </si>
 </sst>
 </file>
@@ -751,25 +754,25 @@
   <sheetData>
     <row r="1" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" t="s">
         <v>101</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -777,7 +780,7 @@
         <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C2" s="1">
         <v>0</v>
@@ -800,7 +803,7 @@
         <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C3" s="1">
         <v>3</v>
@@ -823,7 +826,7 @@
         <v>31</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C4" s="1">
         <v>0</v>
@@ -846,7 +849,7 @@
         <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C5" s="1">
         <v>3</v>
@@ -869,7 +872,7 @@
         <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C6" s="1">
         <v>4</v>
@@ -1102,37 +1105,28 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="B1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C1" t="s">
-        <v>97</v>
-      </c>
-      <c r="D1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
     </row>
-    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
     </row>
-    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
     </row>
   </sheetData>

</xml_diff>